<commit_message>
v11: buying situation in hero, logos up, shorter workflow, sample consistency fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample/ladder-sample-estimate.xlsx
+++ b/sample/ladder-sample-estimate.xlsx
@@ -535,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Riverside Community Library (illustrative) · 90% CD estimate · Rev 2</t>
+          <t>Riverside Community Library (illustrative) · Three-story renovation and addition, 54,000 SF · 90% CD estimate · Rev 2</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t>RFI #7: head height at level 5 not dimensioned</t>
+          <t>RFI #7: head height at level 3 not dimensioned</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1025,47 +1025,32 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RFI numbers continue the project RFI log (#1–#6 already issued by the design team).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Finding</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Action</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>Curtain wall head height at level 5 not dimensioned.</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>A-301</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>RFI #7: confirm head height</t>
         </is>
       </c>
     </row>
@@ -1077,17 +1062,17 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>No existing-conditions survey for interior demolition.</t>
+          <t>Curtain wall head height at level 3 not dimensioned.</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>A-301</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Carried as allowance</t>
+          <t>RFI #7: confirm head height</t>
         </is>
       </c>
     </row>
@@ -1099,39 +1084,39 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Roof drain count missing from plumbing plans.</t>
+          <t>No existing-conditions survey for interior demolition.</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>P-201</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Question to design team</t>
+          <t>Carried as allowance</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Conflict</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Spec calls for phenolic toilet partitions; finish schedule says HDPE.</t>
+          <t>Roof drain count missing from plumbing plans.</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>10 21 13 · A-801</t>
+          <t>P-201</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>RFI #8: confirm material</t>
+          <t>Question to design team</t>
         </is>
       </c>
     </row>
@@ -1143,39 +1128,39 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Hardware set 4 lists closers the door schedule omits.</t>
+          <t>Spec calls for phenolic toilet partitions; finish schedule says HDPE.</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>08 71 00 · A-601</t>
+          <t>10 21 13 · A-801</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>RFI #9: confirm closers</t>
+          <t>RFI #8: confirm material</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Conflict</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Demolition carried as an allowance until the survey arrives.</t>
+          <t>Hardware set 4 lists closers the door schedule omits.</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>02 41 19</t>
+          <t>08 71 00 · A-601</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Stated in basis</t>
+          <t>RFI #9: confirm closers</t>
         </is>
       </c>
     </row>
@@ -1187,15 +1172,37 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
+          <t>Demolition carried as an allowance until the survey arrives.</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>02 41 19</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Stated in basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
           <t>RTU-3 priced at the Addendum 3 size, not the original schedule.</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Add. 3</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Stated in basis</t>
         </is>

</xml_diff>